<commit_message>
record matched dns alignment evidence
Preserve 36 current originals with source and fixture provenance and explicitly record six byte-identical prior images. Freeze round-three blind inputs and prior-response material, retain the round-two disagreement audit, and refresh spreadsheet evidence without revising raw ratings.
</commit_message>
<xml_diff>
--- a/docs/ui-dns-eight/KyDNS-Council.xlsx
+++ b/docs/ui-dns-eight/KyDNS-Council.xlsx
@@ -33859,6 +33859,3590 @@
     <row r="118">
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">7e9df60c4a432ae66a3c069745d4e06db29e2b1b22b4687c762617e5a87121ae</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">70180</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">4907ef9b7573d72d679c78e71914bd1f2552c78786962004f672a57da8953fc9</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">69395</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">0b863dede47be5f8c1f9a5dd791f98066de226edd2feaee4cb3d95c9abed012a</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">39389</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">5b5f0e4a4e902f7e199741a18152d29b2a0c1bf6c40860b58e09ee0bbf541bb8</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">38613</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-blacklists-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">8c05be76d87a2d95329ad72be34f4f9d59a5a6cb6cef7c8609bd5c292ef1b4bb</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">87929</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-blacklists-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">0d36d5bd36dbe8bc524a11dbeef318f9ae95f0198b7c7bc8e9128e600802545d</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">87841</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-blacklists-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">49097122d43542e9d39e98eaebc75dbd8a759d523376f86bc791b2a6d00957f0</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">49491</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-blacklists-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">e37dd1bc34ab325fa129a62a5d365dfa9f8c51c3da62d3eeb967debd16de71f6</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">49709</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dashboard-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">8ecc44b71433cd3e6ffda00c0c152203f34684890b704f6d4ad5c88df3679941</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">57213</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dashboard-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">85a69ee389d3605d8296854f3e0c04abcfed4b18465c8421f6f32fc2e8547778</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">57884</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dashboard-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">5f377ae5aaeda83b90c518a29df474921f561aec84fbd5349323b9b201731d01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">33064</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dashboard-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">343d29d773fea1ab1153ddae343102277e2ddf82df18ee7e58bdda4f93709346</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">33044</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dhcp-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">66eed7bae6c4bc64c7481cf5ee03e12336e3d766e3a36e24584fcab046aa8cdb</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">61434</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dhcp-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">edcecfdaef731e6880905a05df221a56b3c5bbbf5cb404a659a4a04e4341cdf9</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">61639</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dhcp-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">9e69a5ffff89ff1322fa5de6befe1db08f30b35b08d1849b1031e18ae7208497</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">34658</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-dhcp-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">8d5ff3e344221e57caa597b3ba6fd5ccae332053c7073d5ee91198268de6defd</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">34568</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-discovered-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">9fa11071e12df329f9f6d91f9130603d08b8959fc5579c7ccaf5a985c690b345</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">32384</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-discovered-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">9a4eeab9d388923f01f565bf8d9f5eeabff1423a548652fcb6bcbe631a96f512</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">32442</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-discovered-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">4a6775c07e5127b89b92d9bcae7820c1a2f78a2fb54760771f3731bc051d6ef2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">23701</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-discovered-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">035074ab587f2833bcba2127de99831d2a586b60a34539052ec9691864a599bb</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">23217</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-login-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">241b6e89a24135bdd4a7cd9c3c4a23f16244dd950df0d97447e2bac6e874eed6</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">18542</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-login-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">2796b01b26fb74963405e745a1eff3b60cc792d710856c01fb25c32be5f5920f</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">22355</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-login-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">c902022e34f02206b93610bae6da6878f8e3b457b1fdd42ccf8d07470c178695</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">15031</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-login-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">045f4f66bb9dd6e68d605ae2a4ac15517c9977158e9d1634e7e7902d2d0e70cf</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">17915</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-records-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">4763370f654c173ca70224153a7efa544b217966fcaecdb0e4295a2b13f23c44</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">57660</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-records-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">ddcf2ba308363a05a4c6508e8f583bb94ab357a6108b5791c429c3e566044177</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">57667</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-records-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">ea64e4dc4100df47124f0a1968e86141e738399b9cf4c809366662cee15ecfbf</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">34838</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-records-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1b4cf25b1f184e46ed736b08c7da8d48ff45b4ec74506b468fc41e59d69fafd7</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">34420</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-services-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">463ecea9e29d497ca734c4361cca05a9f3c0892ab262710773e03dcb7290d3d0</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">82054</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-services-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">7d7aee66ac1f6ded30269b4181fdc5740b934ce9a9510811db1c9fe4d74f2965</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">81794</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-services-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">ad1d42b294fedec360512978c8ca5e18fc6319908d2c5147dc0d34b156eafb4f</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">33685</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-services-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3f782af35930279b410549b2ae52b5d311b621064efab7630019297c255b9a94</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">33119</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-settings-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">af31d3e944be5406b5425abdd1f6a16606d023bb7d532ff2ae66f3f2ba8c9ddb</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">84909</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-settings-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">a145d1310e3c48812575ca55cf87fa09f767e1349faea2ed115f66fb55147a63</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">84569</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-settings-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">e996a4d7c33e2d8a8ab22124f4b378a62099895e961f11d4b29d66b3e0370b6e</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36060</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-00-before-settings-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3280712b7efd44996e7cfa54d763abb804754a58e224fbaf37371e60ae566479</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">35543</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3c442f4218b6d1d0deef8a61d4bd75fda5f50fd373c2ded5e0ac9c47496b19d6</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">74291</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">b1796624b59ce3350dfd6deda938a45a680b692af2efff1fccb2c7f2bc091aad</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">73519</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">d7a3090005935a90ab537f5a125ee5a814eaee6777f265829008a0bf65343cd4</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">39866</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">189e4ca371bcda0b9f2253a16534648ac666f81a57e33bdf9c511c57039a4502</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">39184</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-blacklists-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">fa54c3007dd680185e85ad516b28b2d843c8216c862295033ae43ef6b0523be4</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">95684</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-blacklists-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3ebbfbe90b77e9a9a1bfd8755f279570ab330ce55eb65aa2c710de145fa2fca1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">95501</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-blacklists-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">613a168b2c65c6a1fad9ab37279680e784e8b33f61976cf17209e5c11409b601</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">56030</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-blacklists-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">7fa75fe96046ba3eecd6ffac5d60759e69bacbff09c9ba8ba1c188cc45d79695</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">56381</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dashboard-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">8aa7ab2bee3c379b811b6428401417f19ac174a4b3a7a5871fff9d88d736696e</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">65014</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dashboard-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">5b44a603bedd2e16ab69bcda75f1f93ab8d3c193e6892823aeaa4946127734dc</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">64970</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dashboard-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">5499843dc81085cf8ce1c00d10a646ecd050d1ca3e24e15e4b8f908b55047b37</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">34636</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dashboard-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6568eabfb54ddb512b9c3419a0e226bb07f6e592e24522e886e1eb3b9482c2b</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">34544</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dhcp-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">011831ab5e3b2d45520afbd090b9f6908bc806515b608f811f5e78bfc219bce8</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">65778</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dhcp-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">9368e0ded383d2a84a97a4bcbb63ae82975b9f4e3ffa2e973bfc57fdb382657d</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">65506</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dhcp-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">f27621162444e21ef2f2df52fce6dbfc6292464099369488026a3c2c7509bd5e</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">35541</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-dhcp-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">5de9a2ad55959650bfa516faf4d13a00536283a15c6e3e52aedd542eabbe9427</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">35427</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-discovered-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">4d2c37e40b541d7eca731aca92db852cf94c6a93c106166ba5b214d3e61ad2ac</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">38091</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-discovered-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3d5ff52ab7a519cfab76484b8c04f1eb1d116e95ab56793af52595a65df6a1ba</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">38301</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-discovered-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">27a7fb4007cbbb9ad6b1b4037f7e7b1e27419dc31b346814a8a9097a8b481cb8</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">24956</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-discovered-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">e0b305420631cdefa47e2b392a555f691bfa90e36f78f6607aac98335c3a1125</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">24654</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-login-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">852570f11b84974f69b8701cdd9fd48782983fa4ded9c46747ae19415ac749a0</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">14652</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-login-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">28ccbf2e360abcb8aa2f22d7b814f362d5dc23ec8c9b07d1d341c473a8bfa39d</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">14837</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-login-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">eb18df452965f9cbf21eddbc6103774cfbc516ec0894f33ee24dfd110f1ec471</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">11801</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-login-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3813c7603cbc757bbbba1ced377cc6989166e5d804859d292798abb052f919f4</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">11874</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-records-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">67f44b63d9b312d8061fe7ac037daaaab96097bec3df422242e35c0c2f461f2b</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">63105</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-records-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">221141fcc0ddf050a760caad549fc35d37c26204a60f45839d3578d26e9ecad8</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">63188</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-records-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">33be50a1b184f84e13e04590f4cf01f9360b09b4ac3ec2dbfb2a260e90514085</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">42122</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-records-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">c9e158b24153aad918eb9decf66c1614dbc9c378863145eed4f937cf3569cddb</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41952</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-services-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">4c50a703c7b78d98ca8f5d07c6819b0b98dcce53f3912bf8c513350d8eac4b59</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">82392</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-services-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">5b0d4af4fb811a36e937db9f6e2972dde50c3aa866850b13399ac51ecb5c1da5</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">82171</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-services-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">12e55272fcbc246e31c094c584b4e9c06f887f65a63beb4f18f40ab6f1792f45</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41905</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-services-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">296d9898bfeec5b922020a585c325dfeb9dc8de707dfceb52b64b3bb13a20a69</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41825</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-settings-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">f91f816d2f4f79b0e398c727ff6dfc4a0c9c813e58bc8fb0ee0b356a0c285dd7</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">66143</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-settings-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">c5dcfdbcba586550edd4374dd10f76044fd14b1765e9207c71ba6e6a1bd23f3a</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">66183</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-settings-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">9c82fa3e9dbcc625754a6d54f9b6c145418c85580cd812c9a8c1b687a4417a49</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36879</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-01-after-settings-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">historical_round2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">c8743a57d2d55a5a2fc58a0edab476b8b7b366a4c80f90e2f9540f5c695d429a</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36426</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3c442f4218b6d1d0deef8a61d4bd75fda5f50fd373c2ded5e0ac9c47496b19d6</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">74291</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">b1796624b59ce3350dfd6deda938a45a680b692af2efff1fccb2c7f2bc091aad</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">73519</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">70ed830cf877fe5f797bf6b20eda4be0b12b167bbd5e0e023278ae46f7f5ef27</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41121</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">a5311fac55631cfe4cbd0b5a54cd0395be8f0fea33e64019cfbbc1f980eee941</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">40467</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-blacklists-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36b665b1347eef4232e5c4157c054949f90ec85b137df069d50790a9203c86c9</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">97304</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-blacklists-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">b45c2ff66bfeb841f40cd8a9065061accc4f863343ae2a37a476b23a3fd5bcf2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">97183</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-blacklists-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">beea4ebdf6cdd5c2e586418d4f890e79246ef7c124c861a64d6a0372edbf985e</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">56702</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-blacklists-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">bd6e02b0c3e2a0128334e5aefa1a57711ace61ca09301467cf50eac377615387</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">56898</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dashboard-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">d4f6f7edaaed356dd28806d90959b9dd92df9215a5501230c91890b94eba5968</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">68960</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dashboard-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">17871d203b3483372d63969b59e7b94f8ae8852df06aaac294adcf9d2a33982f</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">68815</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dashboard-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">af6b4adb1edfa6ac05805d7cbf128fb03b26abcc6604d7e97265e31087ab4dca</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36420</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dashboard-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">77f884974ec45f4f98bb9c517681107b252fdf5958dac2e4e827eeecc27a8c80</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36319</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dhcp-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">c882c2e6dcd4507f373f5061a8e764b2d7203cfd942bcab99f39b927c501355d</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">66502</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dhcp-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">794b841d14612c83ff48591a795c8c34340da81e3a1bc9f54902370256576d79</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">66340</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dhcp-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">017f799337af412bb13e913afcc380072f5c09ced70f93fe0fe7351f430a012b</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36976</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-dhcp-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">bd00189f30962ccd0855ebb4dceddadafbf8c5496002f6766cfd86e9096d3f9e</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">36884</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-discovered-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">5f4c16be5aa4c8cc35665d458ed03bea781962517810854be060a8910b95be28</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">38118</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-discovered-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">d97c166cf5581f84b4300df803de5e4703cf215c0a7213aecccfdd57d90855ed</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">38339</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-discovered-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">9b3215634cc241ee2bd76a34d10660d08f961583b6124d1be67244bd6f6c4177</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">26292</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-discovered-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">f6a9c3d309158d66b19f52dc14c63f54d90c63ccd1571558c3aba007b8002202</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">26208</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-login-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">852570f11b84974f69b8701cdd9fd48782983fa4ded9c46747ae19415ac749a0</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">14652</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-login-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">28ccbf2e360abcb8aa2f22d7b814f362d5dc23ec8c9b07d1d341c473a8bfa39d</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">14837</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-login-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">eb18df452965f9cbf21eddbc6103774cfbc516ec0894f33ee24dfd110f1ec471</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">11801</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-login-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3813c7603cbc757bbbba1ced377cc6989166e5d804859d292798abb052f919f4</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">11874</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-records-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">da94dec616e3bf7ff4a599c02677deda44c9539801b3b841572847d98d242ff4</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">62637</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-records-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">9fbdc2f0f6f670b4fcb0354b26035f8331fb998e4833a7cc6cbed6a7bb5e7809</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">62749</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-records-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">3da8586321d12f65c0222694e0348e1aefa6841256a5e2576581bd6bea158aa0</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41325</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-records-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">375852b00f8a4b5eba0720c3ae518a03bc3899f3230784ceed7e4e966a46a62d</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41140</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-services-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">600e0a5bb1a58348f38efdba1d8740cb3dfd0e3f704fe3068b220891d75fffe8</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">81887</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-services-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">863d95d2169e5fdf97947c9b69ec60fea1e03f41a0ef2e3fed375ef300abd2d5</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">81679</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-services-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">83e11d7b328997d0b3b9ae506fcb788d3f0bfc07c011159c388bdaf6a7c02c04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41450</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-services-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">d9464adfd4d851a54899e5817330a7b914e2e99f7d30957fd7f4a752a855d9cc</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41450</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-settings-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">34ea4e27673aa04011f7669e98cc40987ec6d992cea953bc1027492b986c2ff4</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">66141</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-settings-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">b903652771c3e706cefca41f8448049e3537f16b92b3232502245022e7467131</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">66172</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-settings-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">ef39220b4990261ecf3f55a0bcc657bfacb6ab85614dd68ddff66d189b1a7708</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">38139</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kydns-02-after-settings-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">current_round3</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">816ed0da2af913756719fc83c656c81d3d948927df094f14fc84a2f058807ca2</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">37705</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand-references/kyidentity-02-after-users-manage-desktop-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand_only</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">f13eb7bdc897cf717441dfb5e5ed555efb034eb841fac3bf26f02a7a2de5cfe4</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">92667</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand-references/kyidentity-02-after-users-manage-desktop-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand_only</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">c88074992215e2e10fbb0518cafb30d9043cc434713fff8fdc3de81687a1c873</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">89973</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1280</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand-references/kyidentity-02-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand_only</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">b82cb35eae6ead72c08291c04eb188a7549a84ce2e2cc27e7fd948698c6037b6</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">41497</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand-references/kyidentity-02-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand_only</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">ea7033aea61cc689cc94cb5a362d5c9dd7dfbce798c27ed7ce89e8cbd3198fe1</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">42245</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">844</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">opus-round1.json</t>
         </is>
       </c>
@@ -33878,7 +37462,7 @@
         </is>
       </c>
     </row>
-    <row r="119">
+    <row r="231">
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">sol-round1.json</t>
@@ -33900,7 +37484,7 @@
         </is>
       </c>
     </row>
-    <row r="120">
+    <row r="232">
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">opus-round2.json</t>
@@ -33922,7 +37506,7 @@
         </is>
       </c>
     </row>
-    <row r="121">
+    <row r="233">
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">sol-round2.json</t>

</xml_diff>